<commit_message>
codex continuation: code frozen for the sealed blind-08 (merge check 9 green after a deterministic speed test; closing chain green: strict exit 3 with the approval blockers only, check-register 0, Mac checks 9 PASS)
Progress commit at a major step: the code the blind-08 package is built from. The flaky speed test now tests the promise the scheduler makes (a batch already accounted for when its turn comes is never asked); the cost of a batch asked ahead and covered later stays a recorded trade-off (packet C13). Next: the sealed blind-08 run from a package built from this commit, frozen by hash before the key is opened.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvniLE7s99vdF9mVNC2HLc
</commit_message>
<xml_diff>
--- a/out-drill/a1/a1.xlsx
+++ b/out-drill/a1/a1.xlsx
@@ -550,10 +550,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="285" customHeight="1">
+    <row r="2" ht="300" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>WORKING DRAFT, full register: 205 rows (review status: proposed 205; amendment ops: proposed 44). Rows and ops count as accepted only with a named person's decision bound to their current content. Image readings pending the owner's review: VOL-II-p3-r1, VOL-IV-p6-r1. Validated state: ADD-02; working state ADD-03 is PARTIAL. Pass/fail or scored: contractual_post_award = an obligation under the Project Agreement after award; not assessed at bid stage; pass_fail = a gate checked as met or not met at bid stage (a stated rejection, disqualification, non-responsiveness or exclusion, or a document the VOL-I 11.1 checks require); procedural = a step of the tender process with no stated effect on whether the Proposal stays in; scored = marked under the evaluation criteria (Table 1-1 or the financial evaluation); a shortfall loses marks. 'Change at &lt;stage&gt;' says what that addendum did to the row besides its status (the reading re-made, with its note; dates moved; the ops and annotations, with provision and page); a row whose unit an op reissued or amended elsewhere with the row's own words unchanged reads 'ACTIVE (reissued by &lt;op&gt;, unchanged)'. In 'Text as issued', a segment marked '[&lt;document&gt; &lt;clause&gt; p&lt;n&gt;; issued by ADD-0x]' is that addendum's own text, not text of the volumes as issued. The three state columns: 'Value at the validated stage' says what the row's own quoted words, cells and consequence did across the stages (unchanged, changed, amended with the quoted words unchanged, new, not in force; a deletion and a later reinstatement are both named), with each op that re-reads the row named with its kind and review ('proposed, not accepted'), never counted as a confirmation; 'Interpretation' lists the open issues on the reading (HUMAN DECISION PENDING where a person decides; an applied rule awaiting a person's confirmation; other open issues); 'Approval' says what a person has recorded for the row, its image transcription and every op on its units (an image transcription approval covers the transcription and its displayed translation only, never the interpretation). Evidence codes are defined in the Evidence sheet. Relationship status: confirmed = stated in the documents (the entry quotes the cross-reference), not confirmed by a person; proposed = inferred by a curator or a model, a person decides; possible = a weaker inference.</t>
+          <t>WORKING DRAFT, full register: 205 rows (review status: proposed 205; amendment ops: proposed 44). Rows and ops count as accepted only with a named person's decision bound to their current content. Image readings pending the owner's review: VOL-II-p3-r1, VOL-IV-p6-r1. Validated state: ADD-02; working state ADD-03 is PARTIAL. Pass/fail or scored: contractual_post_award = an obligation under the Project Agreement after award; not assessed at bid stage; pass_fail = a gate checked as met or not met at bid stage (a stated rejection, disqualification, non-responsiveness or exclusion, or a document the VOL-I 11.1 checks require); procedural = a step of the tender process with no stated effect on whether the Proposal stays in; scored = marked under the evaluation criteria (Table 1-1 or the financial evaluation); a shortfall loses marks. 'Change at &lt;stage&gt;' says what that addendum did to the row besides its status (the reading re-made, with its note; dates moved; the ops and annotations, with provision and page); a row whose unit an op reissued or amended elsewhere with the row's own words unchanged reads 'ACTIVE (reissued by &lt;op&gt;, unchanged)'. In 'Text as issued', a segment marked '[&lt;document&gt; &lt;clause&gt; p&lt;n&gt;; issued by ADD-0x]' is that addendum's own text, not text of the volumes as issued. The three state columns: 'Value at the validated stage' says what the row's own quoted words, cells and consequence did across the stages (unchanged, changed, amended with the quoted words unchanged, new, not in force; a deletion and a later reinstatement are both named; at a PARTIAL working state, a row an unresolved provision of ADD-03 names reads 'value in question (unresolved: &lt;provision and reason&gt;)', never 'unchanged'), with each op that re-reads the row named with its kind and review ('proposed, not accepted'), never counted as a confirmation; 'Interpretation' lists the open issues on the reading (HUMAN DECISION PENDING where a person decides; an applied rule awaiting a person's confirmation; other open issues); 'Approval' says what a person has recorded for the row, its image transcription and every op on its units (an image transcription approval covers the transcription and its displayed translation only, never the interpretation). Evidence codes are defined in the Evidence sheet. Relationship status: confirmed = stated in the documents (the entry quotes the cross-reference), not confirmed by a person; proposed = inferred by a curator or a model, a person decides; possible = a weaker inference.</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="AD26" s="4" t="inlineStr">
         <is>
-          <t>changed at ADD-02 by ADD-02/4.1 (the quoted value); value as read: 'ninety-six (96) hours'</t>
+          <t>value in question (unresolved: ADD-03:7.1 unresolved: every op for this provision is invalid); before ADD-03: changed at ADD-02 by ADD-02/4.1 (the quoted value); value as read at ADD-02, in question at ADD-03: 'ninety-six (96) hours'</t>
         </is>
       </c>
       <c r="AE26" s="4" t="inlineStr">
@@ -11251,7 +11251,7 @@
       </c>
       <c r="AD65" s="4" t="inlineStr">
         <is>
-          <t>changed at ADD-02 by ADD-02/2.1 (the quoted value); re-read by ADD-01/Q2 (interprets; proposed, not accepted; not counted as a confirmation); value as read: 'one hundred and fifty (150) pages'</t>
+          <t>value in question (unresolved: ADD-03:Q15 unresolved: no recognised phrasing; a person must write the op or a disposition); before ADD-03: changed at ADD-02 by ADD-02/2.1 (the quoted value); re-read by ADD-01/Q2 (interprets; proposed, not accepted; not counted as a confirmation); value as read at ADD-02, in question at ADD-03: 'one hundred and fifty (150) pages'</t>
         </is>
       </c>
       <c r="AE65" s="4" t="inlineStr">
@@ -21097,7 +21097,7 @@
       </c>
       <c r="AD123" s="4" t="inlineStr">
         <is>
-          <t>unchanged since BASE (unit amended elsewhere at ADD-02 by ADD-02/4.1; the row's words unchanged); value as read: 'Standby provision for all rotating equipment shall be N+1.'</t>
+          <t>value in question (unresolved: ADD-03:7.1 unresolved: every op for this provision is invalid); before ADD-03: unit amended elsewhere at ADD-02 by ADD-02/4.1; the row's words unchanged; value as read at ADD-02, in question at ADD-03: 'Standby provision for all rotating equipment shall be N+1.'</t>
         </is>
       </c>
       <c r="AE123" s="4" t="inlineStr">

</xml_diff>